<commit_message>
save 15 03 2026
</commit_message>
<xml_diff>
--- a/4 четверть_1_HTML_CSS_свойства 1 - шрифт, icons, текст align.xlsx
+++ b/4 четверть_1_HTML_CSS_свойства 1 - шрифт, icons, текст align.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Machenike\Desktop\Homework_repo\GB_Developer_Workbook\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Machenike\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F219A8-43C8-4E89-90A5-188CDF044559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E08FF0A-339D-4186-8369-CA1EECCBC48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" tabRatio="825" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" tabRatio="825" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Названия class" sheetId="24" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="251">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -3571,17 +3571,92 @@
       <t xml:space="preserve"> </t>
     </r>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/* long-hand */</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+font-style: italic;
+font-weight: bold;
+font-size: 15px;
+line-height: 1.2;
+font-family: Arial, sans-serif;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/* short-hand */</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+font:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> italic bold 15px/1.2 Arial, sans-serif;</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -3793,7 +3868,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3830,6 +3905,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -3843,7 +3924,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -3854,20 +3935,20 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -3876,40 +3957,43 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -3918,11 +4002,11 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -3933,16 +4017,16 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4673,12 +4757,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -5262,12 +5346,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -5356,7 +5440,7 @@
       <c r="B8" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="33" t="s">
         <v>249</v>
       </c>
     </row>
@@ -5416,12 +5500,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -5503,7 +5587,7 @@
     <tabColor theme="4" tint="0.39997558519241921"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V45"/>
+  <dimension ref="A1:V46"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -5536,12 +5620,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -5691,226 +5775,232 @@
       </c>
       <c r="C20" s="31"/>
     </row>
-    <row r="21" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A21" s="31"/>
-      <c r="B21" s="31" t="s">
+    <row r="21" spans="1:4" ht="116" x14ac:dyDescent="0.35">
+      <c r="A21" s="2"/>
+      <c r="C21" s="35" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+      <c r="A22" s="31"/>
+      <c r="B22" s="31" t="s">
         <v>215</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C22" s="31" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
+    <row r="23" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="C22" s="31" t="s">
+      <c r="C23" s="31" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
+    <row r="24" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C23" s="31" t="s">
+      <c r="C24" s="31" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
+    <row r="25" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B25" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C24" s="31" t="s">
+      <c r="C25" s="31" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
+    <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="C25" s="31" t="s">
+      <c r="C26" s="31" t="s">
         <v>227</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="87" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
+    <row r="27" spans="1:4" ht="87" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="C26" s="31" t="s">
+      <c r="C27" s="31" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="17" t="s">
+    <row r="28" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="17" t="s">
         <v>236</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="C27" s="31" t="s">
+      <c r="C28" s="31" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="C28" s="31" t="s">
+    <row r="29" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="C29" s="31" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="10" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="10"/>
-    </row>
-    <row r="31" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
+      <c r="B31" s="14"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="10"/>
+    </row>
+    <row r="32" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C32" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="11" t="s">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="13"/>
-    </row>
-    <row r="33" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="13"/>
+    </row>
+    <row r="34" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="C34" s="13" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A34" s="17" t="s">
+    <row r="35" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A35" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="C34" s="13"/>
-    </row>
-    <row r="35" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B35" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>21</v>
-      </c>
+      <c r="C35" s="13"/>
     </row>
     <row r="36" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B36" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B37" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C37" s="13" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C37" s="13" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C38" s="13" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C39" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C40" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" s="10" t="s">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C40" s="13"/>
-      <c r="D40" s="1" t="s">
+      <c r="C41" s="13"/>
+      <c r="D41" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="58" x14ac:dyDescent="0.35">
-      <c r="A41" s="1" t="s">
+    <row r="42" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B42" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C41" s="13" t="s">
+      <c r="C42" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D41" s="19" t="s">
+      <c r="D42" s="19" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="174" x14ac:dyDescent="0.35">
-      <c r="A42" s="1" t="s">
+    <row r="43" spans="1:4" ht="174" x14ac:dyDescent="0.35">
+      <c r="A43" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B42" s="18" t="s">
+      <c r="B43" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="13" t="s">
+      <c r="C43" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="D42" s="19" t="s">
+      <c r="D43" s="19" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="116" x14ac:dyDescent="0.35">
-      <c r="A43" s="1" t="s">
+    <row r="44" spans="1:4" ht="116" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B44" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C43" s="18" t="s">
+      <c r="C44" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="D43" s="19" t="s">
+      <c r="D44" s="19" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A44" s="1" t="s">
+    <row r="45" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A45" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B45" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="18" t="s">
+      <c r="C45" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="D44" s="19" t="s">
+      <c r="D45" s="19" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" s="1" t="s">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
         <v>214</v>
       </c>
     </row>
@@ -5918,7 +6008,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
-  <phoneticPr fontId="22" type="noConversion"/>
+  <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -5964,12 +6054,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -6114,12 +6204,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -6267,12 +6357,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -6403,12 +6493,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.35">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>

</xml_diff>